<commit_message>
Fix dashboard/screener bugs: ROE mean->median (BEL/HAL outlier skew), D/E equals-0 sector exemption, capital allocation null pattern_label filter, peer radar 0-100 normalization
</commit_message>
<xml_diff>
--- a/output/screener_output.xlsx
+++ b/output/screener_output.xlsx
@@ -6092,7 +6092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U19"/>
+  <dimension ref="A1:U3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6228,12 +6228,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>LICI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Punjab National Bank</t>
+          <t>Life Insurance Corporation of India</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -6242,56 +6242,65 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>26.08958669347562</v>
+        <v>69.67912335635215</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>61.32056519118731</v>
+        <v>49.44710986501021</v>
+      </c>
+      <c r="F2" t="n">
+        <v>39.05035832114759</v>
       </c>
       <c r="G2" t="n">
-        <v>8.395910695456838</v>
+        <v>4.836600998148862</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>3.684256345007701</v>
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>371.9375</v>
       </c>
       <c r="K2" t="n">
-        <v>15.90207600910603</v>
+        <v>8.15986061977938</v>
+      </c>
+      <c r="L2" t="n">
+        <v>73.17556747076097</v>
       </c>
       <c r="N2" t="n">
-        <v>-29445</v>
+        <v>853</v>
       </c>
       <c r="O2" t="n">
-        <v>-1.612606778720886</v>
+        <v>0.4646382763782856</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Accrual Risk</t>
+          <t>High Quality</t>
         </is>
       </c>
       <c r="Q2" t="n">
-        <v>19.29</v>
+        <v>30.67</v>
       </c>
       <c r="R2" t="n">
-        <v>10.91</v>
+        <v>8.1</v>
       </c>
       <c r="S2" t="n">
-        <v>1.32</v>
+        <v>3.77</v>
       </c>
       <c r="T2" s="2" t="n">
-        <v>109065</v>
+        <v>845966</v>
       </c>
       <c r="U2" t="n">
-        <v>9157</v>
+        <v>40916</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LICI</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Life Insurance Corporation of India</t>
+          <t>SBI Life Insurance Company Ltd</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6300,34 +6309,37 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>69.67912335635215</v>
+        <v>43.41835827855824</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>49.44710986501021</v>
+        <v>12.70458814059566</v>
       </c>
       <c r="F3" t="n">
-        <v>39.05035832114759</v>
+        <v>1.140327341024953</v>
       </c>
       <c r="G3" t="n">
-        <v>4.836600998148862</v>
+        <v>1.434978937479165</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>371.9375</v>
+        <v>240.3333333333333</v>
       </c>
       <c r="K3" t="n">
-        <v>8.15986061977938</v>
+        <v>24.23161418236754</v>
       </c>
       <c r="L3" t="n">
-        <v>73.17556747076097</v>
+        <v>7.374662152227485</v>
+      </c>
+      <c r="M3" t="n">
+        <v>7.885244396237145</v>
       </c>
       <c r="N3" t="n">
-        <v>853</v>
+        <v>-2099</v>
       </c>
       <c r="O3" t="n">
-        <v>0.4646382763782856</v>
+        <v>-0.2368813254240325</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -6335,1138 +6347,18 @@
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>30.67</v>
+        <v>69.98</v>
       </c>
       <c r="R3" t="n">
-        <v>8.1</v>
+        <v>9.48</v>
       </c>
       <c r="S3" t="n">
-        <v>3.77</v>
+        <v>1.62</v>
       </c>
       <c r="T3" s="2" t="n">
-        <v>845966</v>
+        <v>131988</v>
       </c>
       <c r="U3" t="n">
-        <v>40916</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>PFC</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Power Finance Corporation Ltd</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>27.43053836876541</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>26.1609340860332</v>
-      </c>
-      <c r="F4" t="n">
-        <v>3.480398875307857</v>
-      </c>
-      <c r="G4" t="n">
-        <v>28.91659745596014</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>8.521864217426122</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.5804147544943239</v>
-      </c>
-      <c r="K4" t="n">
-        <v>11.08175357755092</v>
-      </c>
-      <c r="L4" t="n">
-        <v>15.92359362270073</v>
-      </c>
-      <c r="M4" t="n">
-        <v>14.86983549970351</v>
-      </c>
-      <c r="N4" t="n">
-        <v>-101229</v>
-      </c>
-      <c r="O4" t="n">
-        <v>-5.031547988302576</v>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Accrual Risk</t>
-        </is>
-      </c>
-      <c r="Q4" t="n">
-        <v>35.6</v>
-      </c>
-      <c r="R4" t="n">
-        <v>6.59</v>
-      </c>
-      <c r="S4" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="T4" s="2" t="n">
-        <v>91508</v>
-      </c>
-      <c r="U4" t="n">
-        <v>26461</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>BAJAJFINSV</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Bajaj Finserv Ltd</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>25.75641163005052</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>25.85035141227954</v>
-      </c>
-      <c r="F5" t="n">
-        <v>11.44874463510097</v>
-      </c>
-      <c r="G5" t="n">
-        <v>14.12820930948886</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>4.789368120938867</v>
-      </c>
-      <c r="I5" t="n">
-        <v>2.197130112323319</v>
-      </c>
-      <c r="K5" t="n">
-        <v>20.97274568418761</v>
-      </c>
-      <c r="L5" t="n">
-        <v>23.74781614270227</v>
-      </c>
-      <c r="M5" t="n">
-        <v>20.58909506066124</v>
-      </c>
-      <c r="N5" t="n">
-        <v>-79634</v>
-      </c>
-      <c r="O5" t="n">
-        <v>-4.180016339930263</v>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Accrual Risk</t>
-        </is>
-      </c>
-      <c r="Q5" t="n">
-        <v>15.07</v>
-      </c>
-      <c r="R5" t="n">
-        <v>6.08</v>
-      </c>
-      <c r="S5" t="n">
-        <v>2.56</v>
-      </c>
-      <c r="T5" s="2" t="n">
-        <v>110382</v>
-      </c>
-      <c r="U5" t="n">
-        <v>15595</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>RECLTD</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>REC Ltd</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>26.85241957245974</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>20.39653929343908</v>
-      </c>
-      <c r="F6" t="n">
-        <v>9.294489608054098</v>
-      </c>
-      <c r="G6" t="n">
-        <v>29.7682934528695</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>6.424917087238645</v>
-      </c>
-      <c r="I6" t="n">
-        <v>1.600474155202351</v>
-      </c>
-      <c r="K6" t="n">
-        <v>13.33804224786568</v>
-      </c>
-      <c r="L6" t="n">
-        <v>19.76311435023079</v>
-      </c>
-      <c r="M6" t="n">
-        <v>19.67245924901726</v>
-      </c>
-      <c r="N6" t="n">
-        <v>-59554</v>
-      </c>
-      <c r="O6" t="n">
-        <v>-20.40097504287343</v>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Accrual Risk</t>
-        </is>
-      </c>
-      <c r="Q6" t="n">
-        <v>31.49</v>
-      </c>
-      <c r="R6" t="n">
-        <v>4.59</v>
-      </c>
-      <c r="S6" t="n">
-        <v>2.18</v>
-      </c>
-      <c r="T6" s="2" t="n">
-        <v>47517</v>
-      </c>
-      <c r="U6" t="n">
-        <v>14145</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>BAJFINANCE</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Bajaj Finance Ltd</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>33.96649178512514</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>18.8419213518306</v>
-      </c>
-      <c r="F7" t="n">
-        <v>4.166013587646808</v>
-      </c>
-      <c r="G7" t="n">
-        <v>26.28792839991269</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>3.824788776468134</v>
-      </c>
-      <c r="I7" t="n">
-        <v>2689.166666666667</v>
-      </c>
-      <c r="K7" t="n">
-        <v>24.35264273954201</v>
-      </c>
-      <c r="L7" t="n">
-        <v>29.32313482597901</v>
-      </c>
-      <c r="M7" t="n">
-        <v>27.5561392815338</v>
-      </c>
-      <c r="N7" t="n">
-        <v>-79931</v>
-      </c>
-      <c r="O7" t="n">
-        <v>-3.231792280571145</v>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Accrual Risk</t>
-        </is>
-      </c>
-      <c r="Q7" t="n">
-        <v>69.2</v>
-      </c>
-      <c r="R7" t="n">
-        <v>4.11</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="T7" s="2" t="n">
-        <v>54972</v>
-      </c>
-      <c r="U7" t="n">
-        <v>14451</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>ICICIBANK</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>ICICI Bank Ltd</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>55.78104939027111</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>17.99027109750765</v>
-      </c>
-      <c r="F8" t="n">
-        <v>5.11888931768417</v>
-      </c>
-      <c r="G8" t="n">
-        <v>28.8880112339828</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>6.445624336310825</v>
-      </c>
-      <c r="I8" t="n">
-        <v>1.300946133138182</v>
-      </c>
-      <c r="K8" t="n">
-        <v>17.25086850260209</v>
-      </c>
-      <c r="L8" t="n">
-        <v>51.94877118224903</v>
-      </c>
-      <c r="M8" t="n">
-        <v>55.18455739153598</v>
-      </c>
-      <c r="N8" t="n">
-        <v>12547</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0.9510909711578005</v>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>High Quality</t>
-        </is>
-      </c>
-      <c r="Q8" t="n">
-        <v>25.76</v>
-      </c>
-      <c r="R8" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="S8" t="n">
-        <v>3.43</v>
-      </c>
-      <c r="T8" s="2" t="n">
-        <v>159516</v>
-      </c>
-      <c r="U8" t="n">
-        <v>46081</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>CHOLAFIN</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Cholamandalam Investment &amp; Finance Company Ltd</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>26.94888984286409</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>17.45521359669269</v>
-      </c>
-      <c r="F9" t="n">
-        <v>3.366695225484851</v>
-      </c>
-      <c r="G9" t="n">
-        <v>17.84689244899024</v>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>6.863420609401317</v>
-      </c>
-      <c r="I9" t="n">
-        <v>21.21176470588235</v>
-      </c>
-      <c r="K9" t="n">
-        <v>21.93916480497526</v>
-      </c>
-      <c r="L9" t="n">
-        <v>23.36341725167208</v>
-      </c>
-      <c r="M9" t="n">
-        <v>22.27523876455795</v>
-      </c>
-      <c r="N9" t="n">
-        <v>-38538</v>
-      </c>
-      <c r="O9" t="n">
-        <v>-3.965092371280805</v>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>Accrual Risk</t>
-        </is>
-      </c>
-      <c r="Q9" t="n">
-        <v>16.79</v>
-      </c>
-      <c r="R9" t="n">
-        <v>10.36</v>
-      </c>
-      <c r="S9" t="n">
-        <v>2.83</v>
-      </c>
-      <c r="T9" s="2" t="n">
-        <v>19163</v>
-      </c>
-      <c r="U9" t="n">
-        <v>3420</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>CANBK</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Canara Bank</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>50.01209731543244</v>
-      </c>
-      <c r="E10" s="2" t="n">
-        <v>16.71605179468811</v>
-      </c>
-      <c r="F10" t="n">
-        <v>3.09484900948278</v>
-      </c>
-      <c r="G10" t="n">
-        <v>13.93516047014541</v>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>14.86741992554242</v>
-      </c>
-      <c r="I10" t="n">
-        <v>1.610661174334986</v>
-      </c>
-      <c r="K10" t="n">
-        <v>18.17561078322378</v>
-      </c>
-      <c r="L10" t="n">
-        <v>85.7752850068174</v>
-      </c>
-      <c r="M10" t="n">
-        <v>53.4206382524911</v>
-      </c>
-      <c r="N10" t="n">
-        <v>13296</v>
-      </c>
-      <c r="O10" t="n">
-        <v>2.678399409785198</v>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>High Quality</t>
-        </is>
-      </c>
-      <c r="Q10" t="n">
-        <v>36.74</v>
-      </c>
-      <c r="R10" t="n">
-        <v>12.61</v>
-      </c>
-      <c r="S10" t="n">
-        <v>3.81</v>
-      </c>
-      <c r="T10" s="2" t="n">
-        <v>110519</v>
-      </c>
-      <c r="U10" t="n">
-        <v>15401</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>AXISBANK</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Axis Bank Ltd</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>34.78026684048123</v>
-      </c>
-      <c r="E11" s="2" t="n">
-        <v>15.83271240518905</v>
-      </c>
-      <c r="F11" t="n">
-        <v>2.520716781712082</v>
-      </c>
-      <c r="G11" t="n">
-        <v>22.73130411725443</v>
-      </c>
-      <c r="H11" s="2" t="n">
-        <v>8.249122739980766</v>
-      </c>
-      <c r="I11" t="n">
-        <v>1.691203992514036</v>
-      </c>
-      <c r="K11" t="n">
-        <v>14.74358712051438</v>
-      </c>
-      <c r="L11" t="n">
-        <v>39.67228711897934</v>
-      </c>
-      <c r="M11" t="n">
-        <v>35.09600385206135</v>
-      </c>
-      <c r="N11" t="n">
-        <v>-14556</v>
-      </c>
-      <c r="O11" t="n">
-        <v>-1.534037435719632</v>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>High Quality</t>
-        </is>
-      </c>
-      <c r="Q11" t="n">
-        <v>38.14</v>
-      </c>
-      <c r="R11" t="n">
-        <v>4.66</v>
-      </c>
-      <c r="S11" t="n">
-        <v>2.32</v>
-      </c>
-      <c r="T11" s="2" t="n">
-        <v>109369</v>
-      </c>
-      <c r="U11" t="n">
-        <v>24861</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>BANKBARODA</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Bank of Baroda</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>35.98148777373478</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>15.7618637908999</v>
-      </c>
-      <c r="F12" t="n">
-        <v>2.712278690337432</v>
-      </c>
-      <c r="G12" t="n">
-        <v>15.93948250956673</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>12.14371872728943</v>
-      </c>
-      <c r="I12" t="n">
-        <v>1.896747724261721</v>
-      </c>
-      <c r="K12" t="n">
-        <v>17.47729766589094</v>
-      </c>
-      <c r="L12" t="n">
-        <v>74.50588066551305</v>
-      </c>
-      <c r="M12" t="n">
-        <v>55.18455739153598</v>
-      </c>
-      <c r="N12" t="n">
-        <v>-7559</v>
-      </c>
-      <c r="O12" t="n">
-        <v>-1.279081332956056</v>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>High Quality</t>
-        </is>
-      </c>
-      <c r="Q12" t="n">
-        <v>16.89</v>
-      </c>
-      <c r="R12" t="n">
-        <v>4.15</v>
-      </c>
-      <c r="S12" t="n">
-        <v>2.62</v>
-      </c>
-      <c r="T12" s="2" t="n">
-        <v>118379</v>
-      </c>
-      <c r="U12" t="n">
-        <v>18869</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>ICICIGI</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>ICICI Lombard General Insurance Company Ltd</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>57.68825046529937</v>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>15.7230643179025</v>
-      </c>
-      <c r="F13" t="n">
-        <v>145.2287581699346</v>
-      </c>
-      <c r="G13" t="n">
-        <v>9.366915605017816</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>0.002867677181482999</v>
-      </c>
-      <c r="I13" t="n">
-        <v>160.0267857142857</v>
-      </c>
-      <c r="K13" t="n">
-        <v>12.91184100336258</v>
-      </c>
-      <c r="L13" t="n">
-        <v>12.83917371819816</v>
-      </c>
-      <c r="M13" t="n">
-        <v>11.1392224868865</v>
-      </c>
-      <c r="N13" t="n">
-        <v>486</v>
-      </c>
-      <c r="O13" t="n">
-        <v>0.03821387979852416</v>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>High Quality</t>
-        </is>
-      </c>
-      <c r="Q13" t="n">
-        <v>49</v>
-      </c>
-      <c r="R13" t="n">
-        <v>7.86</v>
-      </c>
-      <c r="S13" t="n">
-        <v>3.46</v>
-      </c>
-      <c r="T13" s="2" t="n">
-        <v>20487</v>
-      </c>
-      <c r="U13" t="n">
-        <v>1919</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>SHRIRAMFIN</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Shriram Finance Ltd</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>23.4037502831333</v>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>15.11635033812082</v>
-      </c>
-      <c r="F14" t="n">
-        <v>4.064342198385718</v>
-      </c>
-      <c r="G14" t="n">
-        <v>20.33362647026492</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>3.994034363699512</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0.6766743648960739</v>
-      </c>
-      <c r="K14" t="n">
-        <v>18.55607005277675</v>
-      </c>
-      <c r="L14" t="n">
-        <v>23.49387942502037</v>
-      </c>
-      <c r="M14" t="n">
-        <v>14.28965514115608</v>
-      </c>
-      <c r="N14" t="n">
-        <v>-31359</v>
-      </c>
-      <c r="O14" t="n">
-        <v>-3.608906905151208</v>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>Accrual Risk</t>
-        </is>
-      </c>
-      <c r="Q14" t="n">
-        <v>68.53</v>
-      </c>
-      <c r="R14" t="n">
-        <v>7.91</v>
-      </c>
-      <c r="S14" t="n">
-        <v>1.86</v>
-      </c>
-      <c r="T14" s="2" t="n">
-        <v>36388</v>
-      </c>
-      <c r="U14" t="n">
-        <v>7399</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>HDFCBANK</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>HDFC Bank Ltd</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>46.98858561535396</v>
-      </c>
-      <c r="E15" s="2" t="n">
-        <v>14.33974005030719</v>
-      </c>
-      <c r="F15" t="n">
-        <v>4.801033923800871</v>
-      </c>
-      <c r="G15" t="n">
-        <v>23.07288232992184</v>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>6.808786667718385</v>
-      </c>
-      <c r="I15" t="n">
-        <v>1.400768822479211</v>
-      </c>
-      <c r="K15" t="n">
-        <v>21.95098428169122</v>
-      </c>
-      <c r="L15" t="n">
-        <v>23.86506357287907</v>
-      </c>
-      <c r="M15" t="n">
-        <v>15.42478808253083</v>
-      </c>
-      <c r="N15" t="n">
-        <v>35669</v>
-      </c>
-      <c r="O15" t="n">
-        <v>4.412519521183551</v>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>Accrual Risk</t>
-        </is>
-      </c>
-      <c r="Q15" t="n">
-        <v>49.42</v>
-      </c>
-      <c r="R15" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="S15" t="n">
-        <v>4.33</v>
-      </c>
-      <c r="T15" s="2" t="n">
-        <v>283649</v>
-      </c>
-      <c r="U15" t="n">
-        <v>65446</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>INDUSINDBK</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>IndusInd Bank Ltd</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>28.76228908265894</v>
-      </c>
-      <c r="E16" s="2" t="n">
-        <v>14.25227319776422</v>
-      </c>
-      <c r="F16" t="n">
-        <v>3.475962286021232</v>
-      </c>
-      <c r="G16" t="n">
-        <v>19.56369677362945</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>6.885742949503957</v>
-      </c>
-      <c r="I16" t="n">
-        <v>1.879527055815935</v>
-      </c>
-      <c r="K16" t="n">
-        <v>15.49561308335803</v>
-      </c>
-      <c r="L16" t="n">
-        <v>22.07746495394836</v>
-      </c>
-      <c r="M16" t="n">
-        <v>15.89562187541786</v>
-      </c>
-      <c r="N16" t="n">
-        <v>-17468</v>
-      </c>
-      <c r="O16" t="n">
-        <v>-0.9664534641259643</v>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>High Quality</t>
-        </is>
-      </c>
-      <c r="Q16" t="n">
-        <v>8.99</v>
-      </c>
-      <c r="R16" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="S16" t="n">
-        <v>1.42</v>
-      </c>
-      <c r="T16" s="2" t="n">
-        <v>45748</v>
-      </c>
-      <c r="U16" t="n">
-        <v>8950</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>KOTAKBANK</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Kotak Mahindra Bank Ltd</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>45.85310679979926</v>
-      </c>
-      <c r="E17" s="2" t="n">
-        <v>14.01301818853291</v>
-      </c>
-      <c r="F17" t="n">
-        <v>7.113136699541475</v>
-      </c>
-      <c r="G17" t="n">
-        <v>32.38615146611662</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>4.003739266919029</v>
-      </c>
-      <c r="I17" t="n">
-        <v>1.236375108447038</v>
-      </c>
-      <c r="K17" t="n">
-        <v>13.51960376324537</v>
-      </c>
-      <c r="L17" t="n">
-        <v>20.38200065626572</v>
-      </c>
-      <c r="M17" t="n">
-        <v>19.34407044160125</v>
-      </c>
-      <c r="N17" t="n">
-        <v>6766</v>
-      </c>
-      <c r="O17" t="n">
-        <v>1.572670875827523</v>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>High Quality</t>
-        </is>
-      </c>
-      <c r="Q17" t="n">
-        <v>32.9</v>
-      </c>
-      <c r="R17" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="S17" t="n">
-        <v>1.51</v>
-      </c>
-      <c r="T17" s="2" t="n">
-        <v>56237</v>
-      </c>
-      <c r="U17" t="n">
-        <v>18213</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>IRFC</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Indian Railway Finance Corporation Ltd</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>37.27216186683776</v>
-      </c>
-      <c r="E18" s="2" t="n">
-        <v>13.0380853616381</v>
-      </c>
-      <c r="F18" t="n">
-        <v>5.746523336036321</v>
-      </c>
-      <c r="G18" t="n">
-        <v>24.0645524488647</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>8.378352548852153</v>
-      </c>
-      <c r="I18" t="n">
-        <v>1.31948659270683</v>
-      </c>
-      <c r="K18" t="n">
-        <v>19.06740855567788</v>
-      </c>
-      <c r="L18" t="n">
-        <v>23.24502393394037</v>
-      </c>
-      <c r="M18" t="n">
-        <v>20.11244339814313</v>
-      </c>
-      <c r="N18" t="n">
-        <v>7906</v>
-      </c>
-      <c r="O18" t="n">
-        <v>0.3019460457018293</v>
-      </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>Accrual Risk</t>
-        </is>
-      </c>
-      <c r="Q18" t="n">
-        <v>9.81</v>
-      </c>
-      <c r="R18" t="n">
-        <v>3.91</v>
-      </c>
-      <c r="S18" t="n">
-        <v>2.82</v>
-      </c>
-      <c r="T18" s="2" t="n">
-        <v>26645</v>
-      </c>
-      <c r="U18" t="n">
-        <v>6412</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>SBILIFE</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>SBI Life Insurance Company Ltd</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>43.41835827855824</v>
-      </c>
-      <c r="E19" s="2" t="n">
-        <v>12.70458814059566</v>
-      </c>
-      <c r="F19" t="n">
-        <v>1.140327341024953</v>
-      </c>
-      <c r="G19" t="n">
-        <v>1.434978937479165</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" t="n">
-        <v>240.3333333333333</v>
-      </c>
-      <c r="K19" t="n">
-        <v>24.23161418236754</v>
-      </c>
-      <c r="L19" t="n">
-        <v>7.374662152227485</v>
-      </c>
-      <c r="M19" t="n">
-        <v>7.885244396237145</v>
-      </c>
-      <c r="N19" t="n">
-        <v>-2099</v>
-      </c>
-      <c r="O19" t="n">
-        <v>-0.2368813254240325</v>
-      </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>High Quality</t>
-        </is>
-      </c>
-      <c r="Q19" t="n">
-        <v>69.98</v>
-      </c>
-      <c r="R19" t="n">
-        <v>9.48</v>
-      </c>
-      <c r="S19" t="n">
-        <v>1.62</v>
-      </c>
-      <c r="T19" s="2" t="n">
-        <v>131988</v>
-      </c>
-      <c r="U19" t="n">
         <v>1894</v>
       </c>
     </row>

</xml_diff>